<commit_message>
feat: hospital admin panel and receipt fixes and netlify config
</commit_message>
<xml_diff>
--- a/server/data/Hospital_Patient_Records.xlsx
+++ b/server/data/Hospital_Patient_Records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AM17"/>
+  <dimension ref="A1:AM20"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -559,9 +559,9 @@
         <v>Excel Stored At</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>P10031</v>
+        <v>P10034</v>
       </c>
       <c r="B2" t="str">
         <v>Ramesh Kumar</v>
@@ -582,28 +582,43 @@
         <v>V001</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-10</v>
       </c>
       <c r="I2" t="str">
-        <v>10:51:21</v>
+        <v>10:52:34</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-10</v>
       </c>
       <c r="K2" t="str">
-        <v>10:51:21</v>
+        <v>10:52:34</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-09-09T05:21:22.614Z</v>
+        <v>2026-09-10T05:22:34.672Z</v>
       </c>
       <c r="M2" t="str">
-        <v>2026-09-09T05:21:21.969Z</v>
+        <v>2026-09-10T05:22:34.652Z</v>
       </c>
       <c r="N2" t="str">
-        <v>Patient reported acute symptoms</v>
-      </c>
-      <c r="O2" t="str">
-        <v>45-year-old male presented to the Outpatient Department with primary complaint of Chest Pain / Angina. Clinical evaluation details elicited via adaptive voice/touch intake: Pain / Discomfort Intensity (1-10): 7 / 10 (Severe). Review of prior medical documentation identified: No documented prior chronic morbidities.</v>
+        <v>undefined: undefined</v>
+      </c>
+      <c r="O2" t="str" xml:space="preserve">
+        <v xml:space="preserve">45-year-old male presented to the Ayurvedic Wellness OPD with primary complaint/focus of Chest Pain / Angina. Clinical evaluation details elicited via adaptive voice/touch intake: Pain / Discomfort Intensity (1-10): 7 / 10 (Severe). Allergy Status: No known allergies reported.
+[AYUSH HISTORY - AYURVEDIC ASSESSMENT]
+• Dashavidha Pariksha:
+  - Prakriti (Body Constitution): Vata-Pitta (Active, lean, variable appetite, prefers warmth)
+  - Vikriti (Current Imbalance): Pitta-Vata (Current digestive acidity, restlessness, sleep delay)
+  - Sara (Tissue Quality): Madhyama Sara (Moderate tissue quality, steady vitality)
+  - Samhanana (Body Compactness): Susamhita (Well-compacted, symmetrical bone and muscle build)
+  - Pramana (Body Measurements): Pramana-yukta (Proportionate body dimensions and height)
+  - Satmya (Suitability/Adaptation): Oka-Satmya (Well-adapted to home-cooked wholesome foods)
+  - Sattva (Mental Strength): Madhyama Sattva (Moderate mental resilience and calm focus)
+  - Ahara Shakti (Digestive Capacity): Samagni (Balanced digestive capacity, steady hunger)
+  - Vyayama Shakti (Exercise Capacity): Madhyama Shakti (Moderate physical stamina, walking/yoga)
+  - Vaya (Age Assessment): Madhyama Vaya (Adult, productive age group 20-60 yrs)
+• Ahara Assessment (Diet): Usual Diet: Vegetarian (Wholesome balanced vegetarian meals); Timings: Regular 2-3 times daily (Breakfast, Lunch, Light Dinner); Appetite: Normal, consistent appetite; Water: 2 to 2.5 litres daily, normal/warm water; Tastes: Sweet &amp; Sour (Madhura-Amla), moderately spiced; Digestive Concerns: None / Occasional mild gas after heavy meals.
+• Vihara Assessment (Lifestyle): Routine: Early riser (6:00 AM), structured daily routine; Sleep: Sound 7 hours night sleep, restful awakenings; Exercise: Daily 20-30 min brisk walk or yogasanas; Work/Lifestyle: Desk work with moderate screen exposure; Relaxation: Adequate relaxation, leisure reading / prayer.
+• Ayurvedic Wellness Notes: Preventive wellness and holistic lifestyle rejuvenation assessment. Review of prior medical documentation identified: No documented prior chronic morbidities.</v>
       </c>
       <c r="P2" t="str">
         <v>None explicitly documented in uploaded records</v>
@@ -612,7 +627,7 @@
         <v>None</v>
       </c>
       <c r="R2" t="str">
-        <v>Penicillin / Amoxicillin (No known allergy), NSAIDs (Brufen/Diclofenac) (No known allergy)</v>
+        <v>No Known Drug / Food Allergies (NKDA) (Patient reports no known allergies)</v>
       </c>
       <c r="S2" t="str">
         <v>None</v>
@@ -627,7 +642,7 @@
         <v>No previous diagnostic reports uploaded. Advise baseline investigations as indicated.</v>
       </c>
       <c r="W2" t="str">
-        <v>Attending Doctor</v>
+        <v>Pending Verification</v>
       </c>
       <c r="X2" t="str">
         <v/>
@@ -636,13 +651,13 @@
         <v/>
       </c>
       <c r="Z2" t="str">
-        <v>Verified by Doctor</v>
+        <v>Pending Verification</v>
       </c>
       <c r="AA2" t="str">
-        <v>2026-09-09</v>
+        <v/>
       </c>
       <c r="AB2" t="str">
-        <v>10:52:33</v>
+        <v/>
       </c>
       <c r="AC2" t="str">
         <v>None</v>
@@ -663,27 +678,27 @@
         <v/>
       </c>
       <c r="AI2" t="str">
-        <v>Generated</v>
+        <v>Not Generated</v>
       </c>
       <c r="AJ2" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v/>
       </c>
       <c r="AK2" t="str">
-        <v>http://localhost:5173/receipt/cfb422976dc3b38ed0234ce2239e29236ee66eea7fb8c81a</v>
+        <v/>
       </c>
       <c r="AL2" t="str">
         <v/>
       </c>
       <c r="AM2" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>P10030</v>
+        <v>P10033</v>
       </c>
       <c r="B3" t="str">
-        <v>aman</v>
+        <v>Ramesh Kumar</v>
       </c>
       <c r="C3">
         <v>45</v>
@@ -692,7 +707,7 @@
         <v>MALE</v>
       </c>
       <c r="E3" t="str">
-        <v>3636222</v>
+        <v/>
       </c>
       <c r="F3" t="str">
         <v>Chest Pain / Heaviness</v>
@@ -701,28 +716,43 @@
         <v>V001</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-10</v>
       </c>
       <c r="I3" t="str">
-        <v>21:05:37</v>
+        <v>10:42:31</v>
       </c>
       <c r="J3" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-10</v>
       </c>
       <c r="K3" t="str">
-        <v>21:05:37</v>
+        <v>10:42:31</v>
       </c>
       <c r="L3" t="str">
-        <v>2026-09-07T15:35:37.964Z</v>
+        <v>2026-09-10T05:12:31.804Z</v>
       </c>
       <c r="M3" t="str">
-        <v>2026-09-07T15:35:37.881Z</v>
+        <v>2026-09-10T05:12:31.777Z</v>
       </c>
       <c r="N3" t="str">
-        <v>undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined</v>
-      </c>
-      <c r="O3" t="str">
-        <v>45-year-old male presented to the Outpatient Department with primary complaint of Chest Pain / Angina. Clinical evaluation details elicited via adaptive voice/touch intake: When did the chest pain start?: Not specified; How would you describe the chest pain?: Sharp pricking pain that worsens on deep breathing or coughing; Does the pain spread or radiate anywhere else?: Yes, radiates to Left Arm, Jaw, Neck or Back; What other symptoms are you experiencing together with it?: Profuse cold sweating (Diaphoresis); Pain / Discomfort Intensity (1-10): 7 / 10 (Severe). Review of prior medical documentation identified: No documented prior chronic morbidities.</v>
+        <v>undefined: undefined</v>
+      </c>
+      <c r="O3" t="str" xml:space="preserve">
+        <v xml:space="preserve">45-year-old male presented to the Ayurvedic Wellness OPD with primary complaint/focus of Chest Pain / Angina. Clinical evaluation details elicited via adaptive voice/touch intake: Pain / Discomfort Intensity (1-10): 7 / 10 (Severe). Allergy Status: No known allergies reported.
+[AYUSH HISTORY - AYURVEDIC ASSESSMENT]
+• Dashavidha Pariksha:
+  - Prakriti (Body Constitution): Vata-Pitta (Active, lean, variable appetite, prefers warmth)
+  - Vikriti (Current Imbalance): Pitta-Vata (Current digestive acidity, restlessness, sleep delay)
+  - Sara (Tissue Quality): Madhyama Sara (Moderate tissue quality, steady vitality)
+  - Samhanana (Body Compactness): Susamhita (Well-compacted, symmetrical bone and muscle build)
+  - Pramana (Body Measurements): Pramana-yukta (Proportionate body dimensions and height)
+  - Satmya (Suitability/Adaptation): Oka-Satmya (Well-adapted to home-cooked wholesome foods)
+  - Sattva (Mental Strength): Madhyama Sattva (Moderate mental resilience and calm focus)
+  - Ahara Shakti (Digestive Capacity): Samagni (Balanced digestive capacity, steady hunger)
+  - Vyayama Shakti (Exercise Capacity): Madhyama Shakti (Moderate physical stamina, walking/yoga)
+  - Vaya (Age Assessment): Madhyama Vaya (Adult, productive age group 20-60 yrs)
+• Ahara Assessment (Diet): Usual Diet: Vegetarian (Wholesome balanced vegetarian meals); Timings: Regular 2-3 times daily (Breakfast, Lunch, Light Dinner); Appetite: Normal, consistent appetite; Water: 2 to 2.5 litres daily, normal/warm water; Tastes: Sweet &amp; Sour (Madhura-Amla), moderately spiced; Digestive Concerns: None / Occasional mild gas after heavy meals.
+• Vihara Assessment (Lifestyle): Routine: Early riser (6:00 AM), structured daily routine; Sleep: Sound 7 hours night sleep, restful awakenings; Exercise: Daily 20-30 min brisk walk or yogasanas; Work/Lifestyle: Desk work with moderate screen exposure; Relaxation: Adequate relaxation, leisure reading / prayer.
+• Ayurvedic Wellness Notes: Preventive wellness and holistic lifestyle rejuvenation assessment. Review of prior medical documentation identified: No documented prior chronic morbidities.</v>
       </c>
       <c r="P3" t="str">
         <v>None explicitly documented in uploaded records</v>
@@ -731,10 +761,10 @@
         <v>None</v>
       </c>
       <c r="R3" t="str">
-        <v>Penicillin / Amoxicillin (No known allergy), NSAIDs (Brufen/Diclofenac) (No known allergy)</v>
+        <v>No Known Drug / Food Allergies (NKDA) (Patient reports no known allergies)</v>
       </c>
       <c r="S3" t="str">
-        <v>Patient reports: Yes, radiates to Left Arm, Jaw, Neck or Back. Retrosternal pressure radiating to left arm/jaw with diaphoresis.</v>
+        <v>None</v>
       </c>
       <c r="T3" t="str">
         <v>None</v>
@@ -746,7 +776,7 @@
         <v>No previous diagnostic reports uploaded. Advise baseline investigations as indicated.</v>
       </c>
       <c r="W3" t="str">
-        <v>Dr. S. K. Verma, MD</v>
+        <v>Pending Verification</v>
       </c>
       <c r="X3" t="str">
         <v/>
@@ -755,13 +785,13 @@
         <v/>
       </c>
       <c r="Z3" t="str">
-        <v>Verified by Doctor</v>
+        <v>Pending Verification</v>
       </c>
       <c r="AA3" t="str">
-        <v>2026-09-07</v>
+        <v/>
       </c>
       <c r="AB3" t="str">
-        <v>21:07:10</v>
+        <v/>
       </c>
       <c r="AC3" t="str">
         <v>None</v>
@@ -785,7 +815,7 @@
         <v>Not Generated</v>
       </c>
       <c r="AJ3" t="str">
-        <v>2026-09-07 21:07:10</v>
+        <v/>
       </c>
       <c r="AK3" t="str">
         <v/>
@@ -794,15 +824,15 @@
         <v/>
       </c>
       <c r="AM3" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
-        <v>P10029</v>
+        <v>P10032</v>
       </c>
       <c r="B4" t="str">
-        <v>aman</v>
+        <v>Ramesh Kumar</v>
       </c>
       <c r="C4">
         <v>45</v>
@@ -811,7 +841,7 @@
         <v>MALE</v>
       </c>
       <c r="E4" t="str">
-        <v>3762524241</v>
+        <v/>
       </c>
       <c r="F4" t="str">
         <v>Chest Pain / Heaviness</v>
@@ -820,28 +850,43 @@
         <v>V001</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-10</v>
       </c>
       <c r="I4" t="str">
-        <v>20:46:27</v>
+        <v>10:24:19</v>
       </c>
       <c r="J4" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-10</v>
       </c>
       <c r="K4" t="str">
-        <v>20:46:27</v>
+        <v>10:24:19</v>
       </c>
       <c r="L4" t="str">
-        <v>2026-09-07T15:16:28.138Z</v>
+        <v>2026-09-10T04:54:20.058Z</v>
       </c>
       <c r="M4" t="str">
-        <v>2026-09-07T15:16:27.976Z</v>
+        <v>2026-09-10T04:54:19.409Z</v>
       </c>
       <c r="N4" t="str">
-        <v>undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined</v>
-      </c>
-      <c r="O4" t="str">
-        <v>45-year-old male presented to the Outpatient Department with primary complaint of Chest Pain / Angina. Clinical evaluation details elicited via adaptive voice/touch intake: When did the chest pain start?: Within the last 1-4 hours (Sudden onset); How would you describe the chest pain?: Crushing heavy pressure / tight squeezing sensation; Does the pain spread or radiate anywhere else?: Yes, radiates to Left Arm, Jaw, Neck or Back; What other symptoms are you experiencing together with it?: Profuse cold sweating (Diaphoresis); Pain / Discomfort Intensity (1-10): 7 / 10 (Severe). Review of prior medical documentation identified: No documented prior chronic morbidities.</v>
+        <v>undefined: undefined</v>
+      </c>
+      <c r="O4" t="str" xml:space="preserve">
+        <v xml:space="preserve">45-year-old male presented to the Ayurvedic Wellness OPD with primary complaint/focus of Chest Pain / Angina. Clinical evaluation details elicited via adaptive voice/touch intake: Pain / Discomfort Intensity (1-10): 7 / 10 (Severe). Allergy Status: No known allergies reported.
+[AYUSH HISTORY - AYURVEDIC ASSESSMENT]
+• Dashavidha Pariksha:
+  - Prakriti (Body Constitution): Vata-Pitta (Active, lean, variable appetite, prefers warmth)
+  - Vikriti (Current Imbalance): Pitta-Vata (Current digestive acidity, restlessness, sleep delay)
+  - Sara (Tissue Quality): Madhyama Sara (Moderate tissue quality, steady vitality)
+  - Samhanana (Body Compactness): Susamhita (Well-compacted, symmetrical bone and muscle build)
+  - Pramana (Body Measurements): Pramana-yukta (Proportionate body dimensions and height)
+  - Satmya (Suitability/Adaptation): Oka-Satmya (Well-adapted to home-cooked wholesome foods)
+  - Sattva (Mental Strength): Madhyama Sattva (Moderate mental resilience and calm focus)
+  - Ahara Shakti (Digestive Capacity): Samagni (Balanced digestive capacity, steady hunger)
+  - Vyayama Shakti (Exercise Capacity): Madhyama Shakti (Moderate physical stamina, walking/yoga)
+  - Vaya (Age Assessment): Madhyama Vaya (Adult, productive age group 20-60 yrs)
+• Ahara Assessment (Diet): Usual Diet: Vegetarian (Wholesome balanced vegetarian meals); Timings: Regular 2-3 times daily (Breakfast, Lunch, Light Dinner); Appetite: Normal, consistent appetite; Water: 2 to 2.5 litres daily, normal/warm water; Tastes: Sweet &amp; Sour (Madhura-Amla), moderately spiced; Digestive Concerns: None / Occasional mild gas after heavy meals.
+• Vihara Assessment (Lifestyle): Routine: Early riser (6:00 AM), structured daily routine; Sleep: Sound 7 hours night sleep, restful awakenings; Exercise: Daily 20-30 min brisk walk or yogasanas; Work/Lifestyle: Desk work with moderate screen exposure; Relaxation: Adequate relaxation, leisure reading / prayer.
+• Ayurvedic Wellness Notes: Preventive wellness and holistic lifestyle rejuvenation assessment. Review of prior medical documentation identified: No documented prior chronic morbidities.</v>
       </c>
       <c r="P4" t="str">
         <v>None explicitly documented in uploaded records</v>
@@ -850,10 +895,10 @@
         <v>None</v>
       </c>
       <c r="R4" t="str">
-        <v>Penicillin / Amoxicillin (No known allergy), NSAIDs (Brufen/Diclofenac) (No known allergy)</v>
+        <v>No Known Drug / Food Allergies (NKDA) (Patient reports no known allergies)</v>
       </c>
       <c r="S4" t="str">
-        <v>Patient reports: Crushing heavy pressure / tight squeezing sensation. Retrosternal pressure radiating to left arm/jaw with diaphoresis.; Patient reports: Yes, radiates to Left Arm, Jaw, Neck or Back. Retrosternal pressure radiating to left arm/jaw with diaphoresis.</v>
+        <v>None</v>
       </c>
       <c r="T4" t="str">
         <v>None</v>
@@ -865,7 +910,7 @@
         <v>No previous diagnostic reports uploaded. Advise baseline investigations as indicated.</v>
       </c>
       <c r="W4" t="str">
-        <v>Dr. S. K. Verma, MD</v>
+        <v>Pending Verification</v>
       </c>
       <c r="X4" t="str">
         <v/>
@@ -913,63 +958,63 @@
         <v/>
       </c>
       <c r="AM4" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>P10025</v>
+        <v>P10031</v>
       </c>
       <c r="B5" t="str">
-        <v>Rahul Sharma</v>
+        <v>Ramesh Kumar</v>
       </c>
       <c r="C5">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D5" t="str">
         <v>MALE</v>
       </c>
       <c r="E5" t="str">
-        <v>9876500001</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>Chest Congestion &amp; Cough</v>
+        <v>Chest Pain / Heaviness</v>
       </c>
       <c r="G5" t="str">
         <v>V001</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-07-10</v>
+        <v>2026-09-09</v>
       </c>
       <c r="I5" t="str">
-        <v>15:45:00</v>
+        <v>10:51:21</v>
       </c>
       <c r="J5" t="str">
-        <v>2026-07-10</v>
+        <v>2026-09-09</v>
       </c>
       <c r="K5" t="str">
-        <v>15:45:00</v>
+        <v>10:51:21</v>
       </c>
       <c r="L5" t="str">
-        <v>2026-07-10T10:00:00.000Z</v>
+        <v>2026-09-09T05:21:22.614Z</v>
       </c>
       <c r="M5" t="str">
-        <v>2026-07-10T10:15:00.000Z</v>
+        <v>2026-09-09T05:21:21.969Z</v>
       </c>
       <c r="N5" t="str">
-        <v>undefined: undefined; undefined: undefined</v>
+        <v>Patient reported acute symptoms</v>
       </c>
       <c r="O5" t="str">
-        <v>Patient presented with acute respiratory symptoms now stabilized.</v>
+        <v>45-year-old male presented to the Outpatient Department with primary complaint of Chest Pain / Angina. Clinical evaluation details elicited via adaptive voice/touch intake: Pain / Discomfort Intensity (1-10): 7 / 10 (Severe). Review of prior medical documentation identified: No documented prior chronic morbidities.</v>
       </c>
       <c r="P5" t="str">
-        <v>Seasonal allergic rhinitis</v>
+        <v>None explicitly documented in uploaded records</v>
       </c>
       <c r="Q5" t="str">
-        <v xml:space="preserve">undefined , undefined </v>
+        <v>None</v>
       </c>
       <c r="R5" t="str">
-        <v>None reported (No drug allergies)</v>
+        <v>Penicillin / Amoxicillin (No known allergy), NSAIDs (Brufen/Diclofenac) (No known allergy)</v>
       </c>
       <c r="S5" t="str">
         <v>None</v>
@@ -981,13 +1026,13 @@
         <v>None</v>
       </c>
       <c r="V5" t="str">
-        <v>Patient recovering well from acute bronchitis.</v>
+        <v>No previous diagnostic reports uploaded. Advise baseline investigations as indicated.</v>
       </c>
       <c r="W5" t="str">
-        <v>Dr. S. K. Verma, MD</v>
+        <v>Attending Doctor</v>
       </c>
       <c r="X5" t="str">
-        <v>Patient recovering well from acute bronchitis.</v>
+        <v/>
       </c>
       <c r="Y5" t="str">
         <v/>
@@ -996,25 +1041,25 @@
         <v>Verified by Doctor</v>
       </c>
       <c r="AA5" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-09</v>
       </c>
       <c r="AB5" t="str">
-        <v>21:42:07</v>
+        <v>10:52:33</v>
       </c>
       <c r="AC5" t="str">
-        <v>Amoxicillin 500mg (500mg, 1-0-1, 5 days); Paracetamol 650mg (650mg, SOS, 3 days)</v>
+        <v>None</v>
       </c>
       <c r="AD5" t="str">
-        <v>Amoxicillin 500mg</v>
+        <v>None</v>
       </c>
       <c r="AE5" t="str">
-        <v>500mg</v>
+        <v>-</v>
       </c>
       <c r="AF5" t="str">
-        <v>1-0-1</v>
+        <v>-</v>
       </c>
       <c r="AG5" t="str">
-        <v>After food</v>
+        <v>-</v>
       </c>
       <c r="AH5" t="str">
         <v/>
@@ -1023,10 +1068,10 @@
         <v>Generated</v>
       </c>
       <c r="AJ5" t="str">
-        <v>2026-09-07 21:42:07</v>
+        <v>2026-09-09 10:52:33</v>
       </c>
       <c r="AK5" t="str">
-        <v>http://localhost:5173/receipt/e591c145093f910fe728e9ecef84078bd740ef0ea9c19005</v>
+        <v>http://localhost:5173/receipt/cfb422976dc3b38ed0234ce2239e29236ee66eea7fb8c81a</v>
       </c>
       <c r="AL5" t="str">
         <v/>
@@ -1037,61 +1082,61 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>P10025</v>
+        <v>P10030</v>
       </c>
       <c r="B6" t="str">
-        <v>Rahul Sharma</v>
+        <v>aman</v>
       </c>
       <c r="C6">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D6" t="str">
         <v>MALE</v>
       </c>
       <c r="E6" t="str">
-        <v>9876500001</v>
+        <v>3636222</v>
       </c>
       <c r="F6" t="str">
-        <v>Chest Congestion &amp; Cough</v>
+        <v>Chest Pain / Heaviness</v>
       </c>
       <c r="G6" t="str">
         <v>V001</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-07-10</v>
+        <v>2026-09-07</v>
       </c>
       <c r="I6" t="str">
-        <v>15:45:00</v>
+        <v>21:05:37</v>
       </c>
       <c r="J6" t="str">
-        <v>2026-07-10</v>
+        <v>2026-09-07</v>
       </c>
       <c r="K6" t="str">
-        <v>15:45:00</v>
+        <v>21:05:37</v>
       </c>
       <c r="L6" t="str">
-        <v>2026-07-10T10:00:00.000Z</v>
+        <v>2026-09-07T15:35:37.964Z</v>
       </c>
       <c r="M6" t="str">
-        <v>2026-07-10T10:15:00.000Z</v>
+        <v>2026-09-07T15:35:37.881Z</v>
       </c>
       <c r="N6" t="str">
-        <v>undefined: undefined; undefined: undefined</v>
+        <v>undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined</v>
       </c>
       <c r="O6" t="str">
-        <v>Patient presented with acute respiratory symptoms now stabilized.</v>
+        <v>45-year-old male presented to the Outpatient Department with primary complaint of Chest Pain / Angina. Clinical evaluation details elicited via adaptive voice/touch intake: When did the chest pain start?: Not specified; How would you describe the chest pain?: Sharp pricking pain that worsens on deep breathing or coughing; Does the pain spread or radiate anywhere else?: Yes, radiates to Left Arm, Jaw, Neck or Back; What other symptoms are you experiencing together with it?: Profuse cold sweating (Diaphoresis); Pain / Discomfort Intensity (1-10): 7 / 10 (Severe). Review of prior medical documentation identified: No documented prior chronic morbidities.</v>
       </c>
       <c r="P6" t="str">
-        <v>Seasonal allergic rhinitis</v>
+        <v>None explicitly documented in uploaded records</v>
       </c>
       <c r="Q6" t="str">
-        <v xml:space="preserve">undefined , undefined </v>
+        <v>None</v>
       </c>
       <c r="R6" t="str">
-        <v>None reported (No drug allergies)</v>
+        <v>Penicillin / Amoxicillin (No known allergy), NSAIDs (Brufen/Diclofenac) (No known allergy)</v>
       </c>
       <c r="S6" t="str">
-        <v>None</v>
+        <v>Patient reports: Yes, radiates to Left Arm, Jaw, Neck or Back. Retrosternal pressure radiating to left arm/jaw with diaphoresis.</v>
       </c>
       <c r="T6" t="str">
         <v>None</v>
@@ -1100,13 +1145,13 @@
         <v>None</v>
       </c>
       <c r="V6" t="str">
-        <v>Patient recovering well from acute bronchitis.</v>
+        <v>No previous diagnostic reports uploaded. Advise baseline investigations as indicated.</v>
       </c>
       <c r="W6" t="str">
         <v>Dr. S. K. Verma, MD</v>
       </c>
       <c r="X6" t="str">
-        <v>Patient recovering well from acute bronchitis.</v>
+        <v/>
       </c>
       <c r="Y6" t="str">
         <v/>
@@ -1118,99 +1163,99 @@
         <v>2026-09-07</v>
       </c>
       <c r="AB6" t="str">
-        <v>21:42:07</v>
+        <v>21:07:10</v>
       </c>
       <c r="AC6" t="str">
-        <v>Amoxicillin 500mg (500mg, 1-0-1, 5 days); Paracetamol 650mg (650mg, SOS, 3 days)</v>
+        <v>None</v>
       </c>
       <c r="AD6" t="str">
-        <v>Paracetamol 650mg</v>
+        <v>None</v>
       </c>
       <c r="AE6" t="str">
-        <v>650mg</v>
+        <v>-</v>
       </c>
       <c r="AF6" t="str">
-        <v>SOS</v>
+        <v>-</v>
       </c>
       <c r="AG6" t="str">
-        <v>When fever &gt; 100 F</v>
+        <v>-</v>
       </c>
       <c r="AH6" t="str">
         <v/>
       </c>
       <c r="AI6" t="str">
-        <v>Generated</v>
+        <v>Not Generated</v>
       </c>
       <c r="AJ6" t="str">
-        <v>2026-09-07 21:42:07</v>
+        <v>2026-09-07 21:07:10</v>
       </c>
       <c r="AK6" t="str">
-        <v>http://localhost:5173/receipt/e591c145093f910fe728e9ecef84078bd740ef0ea9c19005</v>
+        <v/>
       </c>
       <c r="AL6" t="str">
         <v/>
       </c>
       <c r="AM6" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>P10025</v>
+        <v>P10029</v>
       </c>
       <c r="B7" t="str">
-        <v>Rahul Sharma</v>
+        <v>aman</v>
       </c>
       <c r="C7">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D7" t="str">
         <v>MALE</v>
       </c>
       <c r="E7" t="str">
-        <v>9876500001</v>
+        <v>3762524241</v>
       </c>
       <c r="F7" t="str">
-        <v>गंभीर सिरदर्द और भारीपन (Severe Throbbing Headache)</v>
+        <v>Chest Pain / Heaviness</v>
       </c>
       <c r="G7" t="str">
-        <v>V002</v>
+        <v>V001</v>
       </c>
       <c r="H7" t="str">
         <v>2026-09-07</v>
       </c>
       <c r="I7" t="str">
-        <v>18:57:43</v>
+        <v>20:46:27</v>
       </c>
       <c r="J7" t="str">
         <v>2026-09-07</v>
       </c>
       <c r="K7" t="str">
-        <v>18:57:43</v>
+        <v>20:46:27</v>
       </c>
       <c r="L7" t="str">
-        <v>2026-07-10T10:00:00.000Z</v>
+        <v>2026-09-07T15:16:28.138Z</v>
       </c>
       <c r="M7" t="str">
-        <v>2026-09-07T13:27:43.120Z</v>
+        <v>2026-09-07T15:16:27.976Z</v>
       </c>
       <c r="N7" t="str">
-        <v>undefined: undefined; undefined: undefined; undefined: undefined</v>
+        <v>undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined</v>
       </c>
       <c r="O7" t="str">
-        <v>25-year-old male returns to OPD (Visit 2). Previous visit on 10 July 2026 for acute bronchitis successfully resolved. Currently presents with acute throbbing headache since 2 days, rated 7/10. Pain is bilateral frontal and temporal, aggravated by digital screens. Denies photophobia, fever, vomiting, neck rigidity, or focal neuro deficits.</v>
+        <v>45-year-old male presented to the Outpatient Department with primary complaint of Chest Pain / Angina. Clinical evaluation details elicited via adaptive voice/touch intake: When did the chest pain start?: Within the last 1-4 hours (Sudden onset); How would you describe the chest pain?: Crushing heavy pressure / tight squeezing sensation; Does the pain spread or radiate anywhere else?: Yes, radiates to Left Arm, Jaw, Neck or Back; What other symptoms are you experiencing together with it?: Profuse cold sweating (Diaphoresis); Pain / Discomfort Intensity (1-10): 7 / 10 (Severe). Review of prior medical documentation identified: No documented prior chronic morbidities.</v>
       </c>
       <c r="P7" t="str">
-        <v>Seasonal allergic rhinitis, Past acute bronchitis (July 2026, resolved)</v>
+        <v>None explicitly documented in uploaded records</v>
       </c>
       <c r="Q7" t="str">
         <v>None</v>
       </c>
       <c r="R7" t="str">
-        <v>Penicillin (Tolerated Amoxyclav in July 2026 without reaction)</v>
+        <v>Penicillin / Amoxicillin (No known allergy), NSAIDs (Brufen/Diclofenac) (No known allergy)</v>
       </c>
       <c r="S7" t="str">
-        <v>None</v>
+        <v>Patient reports: Crushing heavy pressure / tight squeezing sensation. Retrosternal pressure radiating to left arm/jaw with diaphoresis.; Patient reports: Yes, radiates to Left Arm, Jaw, Neck or Back. Retrosternal pressure radiating to left arm/jaw with diaphoresis.</v>
       </c>
       <c r="T7" t="str">
         <v>None</v>
@@ -1219,7 +1264,7 @@
         <v>None</v>
       </c>
       <c r="V7" t="str">
-        <v>BP: 126/82 mmHg. Pulse: 76 bpm. Pupils equal and reactive. Neck supple, no meningeal signs.</v>
+        <v>No previous diagnostic reports uploaded. Advise baseline investigations as indicated.</v>
       </c>
       <c r="W7" t="str">
         <v>Dr. S. K. Verma, MD</v>
@@ -1240,19 +1285,19 @@
         <v/>
       </c>
       <c r="AC7" t="str">
-        <v>Naproxen (250 mg, Twice daily SOS (1-0-1), 3 days); Tab Pantoprazole (40 mg, Once daily morning (1-0-0), 5 days)</v>
+        <v>None</v>
       </c>
       <c r="AD7" t="str">
-        <v>Naproxen</v>
+        <v>None</v>
       </c>
       <c r="AE7" t="str">
-        <v>250 mg</v>
+        <v>-</v>
       </c>
       <c r="AF7" t="str">
-        <v>Twice daily SOS (1-0-1)</v>
+        <v>-</v>
       </c>
       <c r="AG7" t="str">
-        <v>Take strictly after meals with antacid</v>
+        <v>-</v>
       </c>
       <c r="AH7" t="str">
         <v/>
@@ -1270,7 +1315,7 @@
         <v/>
       </c>
       <c r="AM7" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
     <row r="8">
@@ -1290,43 +1335,43 @@
         <v>9876500001</v>
       </c>
       <c r="F8" t="str">
-        <v>गंभीर सिरदर्द और भारीपन (Severe Throbbing Headache)</v>
+        <v>Chest Congestion &amp; Cough</v>
       </c>
       <c r="G8" t="str">
-        <v>V002</v>
+        <v>V001</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-09-07</v>
+        <v>2026-07-10</v>
       </c>
       <c r="I8" t="str">
-        <v>18:57:43</v>
+        <v>15:45:00</v>
       </c>
       <c r="J8" t="str">
-        <v>2026-09-07</v>
+        <v>2026-07-10</v>
       </c>
       <c r="K8" t="str">
-        <v>18:57:43</v>
+        <v>15:45:00</v>
       </c>
       <c r="L8" t="str">
         <v>2026-07-10T10:00:00.000Z</v>
       </c>
       <c r="M8" t="str">
-        <v>2026-09-07T13:27:43.120Z</v>
+        <v>2026-07-10T10:15:00.000Z</v>
       </c>
       <c r="N8" t="str">
-        <v>undefined: undefined; undefined: undefined; undefined: undefined</v>
+        <v>undefined: undefined; undefined: undefined</v>
       </c>
       <c r="O8" t="str">
-        <v>25-year-old male returns to OPD (Visit 2). Previous visit on 10 July 2026 for acute bronchitis successfully resolved. Currently presents with acute throbbing headache since 2 days, rated 7/10. Pain is bilateral frontal and temporal, aggravated by digital screens. Denies photophobia, fever, vomiting, neck rigidity, or focal neuro deficits.</v>
+        <v>Patient presented with acute respiratory symptoms now stabilized.</v>
       </c>
       <c r="P8" t="str">
-        <v>Seasonal allergic rhinitis, Past acute bronchitis (July 2026, resolved)</v>
+        <v>Seasonal allergic rhinitis</v>
       </c>
       <c r="Q8" t="str">
-        <v>None</v>
+        <v xml:space="preserve">undefined , undefined </v>
       </c>
       <c r="R8" t="str">
-        <v>Penicillin (Tolerated Amoxyclav in July 2026 without reaction)</v>
+        <v>None reported (No drug allergies)</v>
       </c>
       <c r="S8" t="str">
         <v>None</v>
@@ -1338,132 +1383,132 @@
         <v>None</v>
       </c>
       <c r="V8" t="str">
-        <v>BP: 126/82 mmHg. Pulse: 76 bpm. Pupils equal and reactive. Neck supple, no meningeal signs.</v>
+        <v>Patient recovering well from acute bronchitis.</v>
       </c>
       <c r="W8" t="str">
         <v>Dr. S. K. Verma, MD</v>
       </c>
       <c r="X8" t="str">
-        <v/>
+        <v>Patient recovering well from acute bronchitis.</v>
       </c>
       <c r="Y8" t="str">
         <v/>
       </c>
       <c r="Z8" t="str">
-        <v>Pending Verification</v>
+        <v>Verified by Doctor</v>
       </c>
       <c r="AA8" t="str">
-        <v/>
+        <v>2026-09-07</v>
       </c>
       <c r="AB8" t="str">
-        <v/>
+        <v>21:42:07</v>
       </c>
       <c r="AC8" t="str">
-        <v>Naproxen (250 mg, Twice daily SOS (1-0-1), 3 days); Tab Pantoprazole (40 mg, Once daily morning (1-0-0), 5 days)</v>
+        <v>Amoxicillin 500mg (500mg, 1-0-1, 5 days); Paracetamol 650mg (650mg, SOS, 3 days)</v>
       </c>
       <c r="AD8" t="str">
-        <v>Tab Pantoprazole</v>
+        <v>Amoxicillin 500mg</v>
       </c>
       <c r="AE8" t="str">
-        <v>40 mg</v>
+        <v>500mg</v>
       </c>
       <c r="AF8" t="str">
-        <v>Once daily morning (1-0-0)</v>
+        <v>1-0-1</v>
       </c>
       <c r="AG8" t="str">
-        <v>Take empty stomach before breakfast</v>
+        <v>After food</v>
       </c>
       <c r="AH8" t="str">
         <v/>
       </c>
       <c r="AI8" t="str">
-        <v>Not Generated</v>
+        <v>Generated</v>
       </c>
       <c r="AJ8" t="str">
-        <v/>
+        <v>2026-09-07 21:42:07</v>
       </c>
       <c r="AK8" t="str">
-        <v/>
+        <v>http://localhost:5173/receipt/e591c145093f910fe728e9ecef84078bd740ef0ea9c19005</v>
       </c>
       <c r="AL8" t="str">
         <v/>
       </c>
       <c r="AM8" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>P10026</v>
+        <v>P10025</v>
       </c>
       <c r="B9" t="str">
-        <v>Ramesh Kumar</v>
+        <v>Rahul Sharma</v>
       </c>
       <c r="C9">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="D9" t="str">
         <v>MALE</v>
       </c>
       <c r="E9" t="str">
-        <v>9876543210</v>
+        <v>9876500001</v>
       </c>
       <c r="F9" t="str">
-        <v>डायबिटीज और बीपी चेकअप (Diabetes &amp; BP Follow-up)</v>
+        <v>Chest Congestion &amp; Cough</v>
       </c>
       <c r="G9" t="str">
         <v>V001</v>
       </c>
       <c r="H9" t="str">
-        <v>2025-11-15</v>
+        <v>2026-07-10</v>
       </c>
       <c r="I9" t="str">
-        <v>15:00:00</v>
+        <v>15:45:00</v>
       </c>
       <c r="J9" t="str">
-        <v>2025-11-15</v>
+        <v>2026-07-10</v>
       </c>
       <c r="K9" t="str">
-        <v>15:00:00</v>
+        <v>15:45:00</v>
       </c>
       <c r="L9" t="str">
-        <v>2025-11-15T09:00:00.000Z</v>
+        <v>2026-07-10T10:00:00.000Z</v>
       </c>
       <c r="M9" t="str">
-        <v>2025-11-15T09:30:00.000Z</v>
+        <v>2026-07-10T10:15:00.000Z</v>
       </c>
       <c r="N9" t="str">
-        <v>रूटीन 3 महीने का चेकअप और दवाओं का रीफिल।</v>
+        <v>undefined: undefined; undefined: undefined</v>
       </c>
       <c r="O9" t="str">
-        <v>58-year-old male attended for chronic disease monitoring. Reports compliance with oral hypoglycemics and antihypertensives. Recent HbA1c 8.8%.</v>
+        <v>Patient presented with acute respiratory symptoms now stabilized.</v>
       </c>
       <c r="P9" t="str">
-        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2)</v>
+        <v>Seasonal allergic rhinitis</v>
       </c>
       <c r="Q9" t="str">
-        <v>Metformin 500 mg, Telmisartan 40 mg, Atorvastatin 20 mg, Aspirin (Enteric Coated) 75 mg</v>
+        <v xml:space="preserve">undefined , undefined </v>
       </c>
       <c r="R9" t="str">
-        <v>Penicillin (No known adverse reaction)</v>
+        <v>None reported (No drug allergies)</v>
       </c>
       <c r="S9" t="str">
         <v>None</v>
       </c>
       <c r="T9" t="str">
-        <v>District_Civil_Hospital_Prescription_Nov2025.jpg (prescription)</v>
+        <v>None</v>
       </c>
       <c r="U9" t="str">
         <v>None</v>
       </c>
       <c r="V9" t="str">
-        <v>HbA1c: 8.8%. BP: 154/96 mmHg. Prescribed triple therapy.</v>
+        <v>Patient recovering well from acute bronchitis.</v>
       </c>
       <c r="W9" t="str">
-        <v>Dr. A. Gupta, MD</v>
+        <v>Dr. S. K. Verma, MD</v>
       </c>
       <c r="X9" t="str">
-        <v>Glycemic control suboptimal (HbA1c 8.8%). Advised dietary moderation and continued compliance.</v>
+        <v>Patient recovering well from acute bronchitis.</v>
       </c>
       <c r="Y9" t="str">
         <v/>
@@ -1472,117 +1517,117 @@
         <v>Verified by Doctor</v>
       </c>
       <c r="AA9" t="str">
-        <v>2025-11-15</v>
+        <v>2026-09-07</v>
       </c>
       <c r="AB9" t="str">
-        <v>15:30:00</v>
+        <v>21:42:07</v>
       </c>
       <c r="AC9" t="str">
-        <v>Telmisartan (40 mg, Once daily morning (1-0-0), 90 days); Metformin (500 mg, Twice daily (1-0-1), 90 days); Atorvastatin (20 mg, Once daily bedtime (0-0-1), 90 days)</v>
+        <v>Amoxicillin 500mg (500mg, 1-0-1, 5 days); Paracetamol 650mg (650mg, SOS, 3 days)</v>
       </c>
       <c r="AD9" t="str">
-        <v>Telmisartan</v>
+        <v>Paracetamol 650mg</v>
       </c>
       <c r="AE9" t="str">
-        <v>40 mg</v>
+        <v>650mg</v>
       </c>
       <c r="AF9" t="str">
-        <v>Once daily morning (1-0-0)</v>
+        <v>SOS</v>
       </c>
       <c r="AG9" t="str">
-        <v>Take in morning with water for blood pressure</v>
+        <v>When fever &gt; 100 F</v>
       </c>
       <c r="AH9" t="str">
         <v/>
       </c>
       <c r="AI9" t="str">
-        <v>Not Generated</v>
+        <v>Generated</v>
       </c>
       <c r="AJ9" t="str">
-        <v>2025-11-15 15:30:00</v>
+        <v>2026-09-07 21:42:07</v>
       </c>
       <c r="AK9" t="str">
-        <v/>
+        <v>http://localhost:5173/receipt/e591c145093f910fe728e9ecef84078bd740ef0ea9c19005</v>
       </c>
       <c r="AL9" t="str">
         <v/>
       </c>
       <c r="AM9" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>P10026</v>
+        <v>P10025</v>
       </c>
       <c r="B10" t="str">
-        <v>Ramesh Kumar</v>
+        <v>Rahul Sharma</v>
       </c>
       <c r="C10">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="D10" t="str">
         <v>MALE</v>
       </c>
       <c r="E10" t="str">
-        <v>9876543210</v>
+        <v>9876500001</v>
       </c>
       <c r="F10" t="str">
-        <v>डायबिटीज और बीपी चेकअप (Diabetes &amp; BP Follow-up)</v>
+        <v>गंभीर सिरदर्द और भारीपन (Severe Throbbing Headache)</v>
       </c>
       <c r="G10" t="str">
-        <v>V001</v>
+        <v>V002</v>
       </c>
       <c r="H10" t="str">
-        <v>2025-11-15</v>
+        <v>2026-09-07</v>
       </c>
       <c r="I10" t="str">
-        <v>15:00:00</v>
+        <v>18:57:43</v>
       </c>
       <c r="J10" t="str">
-        <v>2025-11-15</v>
+        <v>2026-09-07</v>
       </c>
       <c r="K10" t="str">
-        <v>15:00:00</v>
+        <v>18:57:43</v>
       </c>
       <c r="L10" t="str">
-        <v>2025-11-15T09:00:00.000Z</v>
+        <v>2026-07-10T10:00:00.000Z</v>
       </c>
       <c r="M10" t="str">
-        <v>2025-11-15T09:30:00.000Z</v>
+        <v>2026-09-07T13:27:43.120Z</v>
       </c>
       <c r="N10" t="str">
-        <v>रूटीन 3 महीने का चेकअप और दवाओं का रीफिल।</v>
+        <v>undefined: undefined; undefined: undefined; undefined: undefined</v>
       </c>
       <c r="O10" t="str">
-        <v>58-year-old male attended for chronic disease monitoring. Reports compliance with oral hypoglycemics and antihypertensives. Recent HbA1c 8.8%.</v>
+        <v>25-year-old male returns to OPD (Visit 2). Previous visit on 10 July 2026 for acute bronchitis successfully resolved. Currently presents with acute throbbing headache since 2 days, rated 7/10. Pain is bilateral frontal and temporal, aggravated by digital screens. Denies photophobia, fever, vomiting, neck rigidity, or focal neuro deficits.</v>
       </c>
       <c r="P10" t="str">
-        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2)</v>
+        <v>Seasonal allergic rhinitis, Past acute bronchitis (July 2026, resolved)</v>
       </c>
       <c r="Q10" t="str">
-        <v>Metformin 500 mg, Telmisartan 40 mg, Atorvastatin 20 mg, Aspirin (Enteric Coated) 75 mg</v>
+        <v xml:space="preserve">undefined , undefined </v>
       </c>
       <c r="R10" t="str">
-        <v>Penicillin (No known adverse reaction)</v>
+        <v>Penicillin (Tolerated Amoxyclav in July 2026 without reaction)</v>
       </c>
       <c r="S10" t="str">
         <v>None</v>
       </c>
       <c r="T10" t="str">
-        <v>District_Civil_Hospital_Prescription_Nov2025.jpg (prescription)</v>
+        <v>None</v>
       </c>
       <c r="U10" t="str">
         <v>None</v>
       </c>
       <c r="V10" t="str">
-        <v>HbA1c: 8.8%. BP: 154/96 mmHg. Prescribed triple therapy.</v>
+        <v>BP: 126/82 mmHg. Pulse: 76 bpm. Pupils equal and reactive. Neck supple, no meningeal signs.</v>
       </c>
       <c r="W10" t="str">
-        <v>Dr. A. Gupta, MD</v>
+        <v>Dr. S. K. Verma, MD</v>
       </c>
       <c r="X10" t="str">
-        <v>Glycemic control suboptimal (HbA1c 8.8%). Advised dietary moderation and continued compliance.</v>
+        <v/>
       </c>
       <c r="Y10" t="str">
         <v/>
@@ -1591,117 +1636,117 @@
         <v>Verified by Doctor</v>
       </c>
       <c r="AA10" t="str">
-        <v>2025-11-15</v>
+        <v>2026-09-10</v>
       </c>
       <c r="AB10" t="str">
-        <v>15:30:00</v>
+        <v>10:44:47</v>
       </c>
       <c r="AC10" t="str">
-        <v>Telmisartan (40 mg, Once daily morning (1-0-0), 90 days); Metformin (500 mg, Twice daily (1-0-1), 90 days); Atorvastatin (20 mg, Once daily bedtime (0-0-1), 90 days)</v>
+        <v>Naproxen (250 mg, Twice daily SOS (1-0-1), 3 days); Tab Pantoprazole (40 mg, Once daily morning (1-0-0), 5 days)</v>
       </c>
       <c r="AD10" t="str">
-        <v>Metformin</v>
+        <v>Naproxen</v>
       </c>
       <c r="AE10" t="str">
-        <v>500 mg</v>
+        <v>250 mg</v>
       </c>
       <c r="AF10" t="str">
-        <v>Twice daily (1-0-1)</v>
+        <v>Twice daily SOS (1-0-1)</v>
       </c>
       <c r="AG10" t="str">
-        <v>Take after breakfast and dinner for blood sugar</v>
+        <v>Take strictly after meals with antacid</v>
       </c>
       <c r="AH10" t="str">
         <v/>
       </c>
       <c r="AI10" t="str">
-        <v>Not Generated</v>
+        <v>Generated</v>
       </c>
       <c r="AJ10" t="str">
-        <v>2025-11-15 15:30:00</v>
+        <v>2026-09-10 10:44:47</v>
       </c>
       <c r="AK10" t="str">
-        <v/>
+        <v>http://localhost:5173/receipt/eb14e62b169c580f0aeefa1fec8a6ccc8362d31e914f8780</v>
       </c>
       <c r="AL10" t="str">
         <v/>
       </c>
       <c r="AM10" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:44:47</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>P10026</v>
+        <v>P10025</v>
       </c>
       <c r="B11" t="str">
-        <v>Ramesh Kumar</v>
+        <v>Rahul Sharma</v>
       </c>
       <c r="C11">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="D11" t="str">
         <v>MALE</v>
       </c>
       <c r="E11" t="str">
-        <v>9876543210</v>
+        <v>9876500001</v>
       </c>
       <c r="F11" t="str">
-        <v>डायबिटीज और बीपी चेकअप (Diabetes &amp; BP Follow-up)</v>
+        <v>गंभीर सिरदर्द और भारीपन (Severe Throbbing Headache)</v>
       </c>
       <c r="G11" t="str">
-        <v>V001</v>
+        <v>V002</v>
       </c>
       <c r="H11" t="str">
-        <v>2025-11-15</v>
+        <v>2026-09-07</v>
       </c>
       <c r="I11" t="str">
-        <v>15:00:00</v>
+        <v>18:57:43</v>
       </c>
       <c r="J11" t="str">
-        <v>2025-11-15</v>
+        <v>2026-09-07</v>
       </c>
       <c r="K11" t="str">
-        <v>15:00:00</v>
+        <v>18:57:43</v>
       </c>
       <c r="L11" t="str">
-        <v>2025-11-15T09:00:00.000Z</v>
+        <v>2026-07-10T10:00:00.000Z</v>
       </c>
       <c r="M11" t="str">
-        <v>2025-11-15T09:30:00.000Z</v>
+        <v>2026-09-07T13:27:43.120Z</v>
       </c>
       <c r="N11" t="str">
-        <v>रूटीन 3 महीने का चेकअप और दवाओं का रीफिल।</v>
+        <v>undefined: undefined; undefined: undefined; undefined: undefined</v>
       </c>
       <c r="O11" t="str">
-        <v>58-year-old male attended for chronic disease monitoring. Reports compliance with oral hypoglycemics and antihypertensives. Recent HbA1c 8.8%.</v>
+        <v>25-year-old male returns to OPD (Visit 2). Previous visit on 10 July 2026 for acute bronchitis successfully resolved. Currently presents with acute throbbing headache since 2 days, rated 7/10. Pain is bilateral frontal and temporal, aggravated by digital screens. Denies photophobia, fever, vomiting, neck rigidity, or focal neuro deficits.</v>
       </c>
       <c r="P11" t="str">
-        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2)</v>
+        <v>Seasonal allergic rhinitis, Past acute bronchitis (July 2026, resolved)</v>
       </c>
       <c r="Q11" t="str">
-        <v>Metformin 500 mg, Telmisartan 40 mg, Atorvastatin 20 mg, Aspirin (Enteric Coated) 75 mg</v>
+        <v xml:space="preserve">undefined , undefined </v>
       </c>
       <c r="R11" t="str">
-        <v>Penicillin (No known adverse reaction)</v>
+        <v>Penicillin (Tolerated Amoxyclav in July 2026 without reaction)</v>
       </c>
       <c r="S11" t="str">
         <v>None</v>
       </c>
       <c r="T11" t="str">
-        <v>District_Civil_Hospital_Prescription_Nov2025.jpg (prescription)</v>
+        <v>None</v>
       </c>
       <c r="U11" t="str">
         <v>None</v>
       </c>
       <c r="V11" t="str">
-        <v>HbA1c: 8.8%. BP: 154/96 mmHg. Prescribed triple therapy.</v>
+        <v>BP: 126/82 mmHg. Pulse: 76 bpm. Pupils equal and reactive. Neck supple, no meningeal signs.</v>
       </c>
       <c r="W11" t="str">
-        <v>Dr. A. Gupta, MD</v>
+        <v>Dr. S. K. Verma, MD</v>
       </c>
       <c r="X11" t="str">
-        <v>Glycemic control suboptimal (HbA1c 8.8%). Advised dietary moderation and continued compliance.</v>
+        <v/>
       </c>
       <c r="Y11" t="str">
         <v/>
@@ -1710,43 +1755,43 @@
         <v>Verified by Doctor</v>
       </c>
       <c r="AA11" t="str">
-        <v>2025-11-15</v>
+        <v>2026-09-10</v>
       </c>
       <c r="AB11" t="str">
-        <v>15:30:00</v>
+        <v>10:44:47</v>
       </c>
       <c r="AC11" t="str">
-        <v>Telmisartan (40 mg, Once daily morning (1-0-0), 90 days); Metformin (500 mg, Twice daily (1-0-1), 90 days); Atorvastatin (20 mg, Once daily bedtime (0-0-1), 90 days)</v>
+        <v>Naproxen (250 mg, Twice daily SOS (1-0-1), 3 days); Tab Pantoprazole (40 mg, Once daily morning (1-0-0), 5 days)</v>
       </c>
       <c r="AD11" t="str">
-        <v>Atorvastatin</v>
+        <v>Tab Pantoprazole</v>
       </c>
       <c r="AE11" t="str">
-        <v>20 mg</v>
+        <v>40 mg</v>
       </c>
       <c r="AF11" t="str">
-        <v>Once daily bedtime (0-0-1)</v>
+        <v>Once daily morning (1-0-0)</v>
       </c>
       <c r="AG11" t="str">
-        <v>Take at night for cholesterol control</v>
+        <v>Take empty stomach before breakfast</v>
       </c>
       <c r="AH11" t="str">
         <v/>
       </c>
       <c r="AI11" t="str">
-        <v>Not Generated</v>
+        <v>Generated</v>
       </c>
       <c r="AJ11" t="str">
-        <v>2025-11-15 15:30:00</v>
+        <v>2026-09-10 10:44:47</v>
       </c>
       <c r="AK11" t="str">
-        <v/>
+        <v>http://localhost:5173/receipt/eb14e62b169c580f0aeefa1fec8a6ccc8362d31e914f8780</v>
       </c>
       <c r="AL11" t="str">
         <v/>
       </c>
       <c r="AM11" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:44:47</v>
       </c>
     </row>
     <row r="12">
@@ -1766,46 +1811,46 @@
         <v>9876543210</v>
       </c>
       <c r="F12" t="str">
-        <v>सीने में भारीपन व पसीना (Acute Chest Heaviness)</v>
+        <v>डायबिटीज और बीपी चेकअप (Diabetes &amp; BP Follow-up)</v>
       </c>
       <c r="G12" t="str">
-        <v>V002</v>
+        <v>V001</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-09-07</v>
+        <v>2025-11-15</v>
       </c>
       <c r="I12" t="str">
-        <v>19:32:43</v>
+        <v>15:00:00</v>
       </c>
       <c r="J12" t="str">
-        <v>2026-09-07</v>
+        <v>2025-11-15</v>
       </c>
       <c r="K12" t="str">
-        <v>19:32:43</v>
+        <v>15:00:00</v>
       </c>
       <c r="L12" t="str">
         <v>2025-11-15T09:00:00.000Z</v>
       </c>
       <c r="M12" t="str">
-        <v>2026-09-07T14:02:43.134Z</v>
+        <v>2025-11-15T09:30:00.000Z</v>
       </c>
       <c r="N12" t="str">
-        <v>undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined</v>
+        <v>रूटीन 3 महीने का चेकअप और दवाओं का रीफिल।</v>
       </c>
       <c r="O12" t="str">
-        <v>58-year-old male with prior hospital records (Visit 1, Nov 2025 for T2DM/HTN) returns with sudden onset crushing retrosternal chest heaviness since 2 hours. Pain radiates to left arm and shoulder, associated with severe cold diaphoresis. Prior medications documented: Metformin 500mg BD, Telmisartan 40mg OD, Atorvastatin 20mg HS.</v>
+        <v>58-year-old male attended for chronic disease monitoring. Reports compliance with oral hypoglycemics and antihypertensives. Recent HbA1c 8.8%.</v>
       </c>
       <c r="P12" t="str">
-        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2), Mixed Dyslipidemia</v>
+        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2)</v>
       </c>
       <c r="Q12" t="str">
         <v>Metformin 500 mg, Telmisartan 40 mg, Atorvastatin 20 mg, Aspirin (Enteric Coated) 75 mg</v>
       </c>
       <c r="R12" t="str">
-        <v>Penicillin (No known allergy)</v>
+        <v>Penicillin (No known adverse reaction)</v>
       </c>
       <c r="S12" t="str">
-        <v>Crushing retrosternal chest pain of acute onset radiating to left arm with profuse cold diaphoresis.; History of Uncontrolled Type 2 Diabetes (HbA1c 8.8%) and Essential Hypertension (BP 154/96 recorded in Nov 2025 visit).</v>
+        <v>None</v>
       </c>
       <c r="T12" t="str">
         <v>District_Civil_Hospital_Prescription_Nov2025.jpg (prescription)</v>
@@ -1814,40 +1859,40 @@
         <v>None</v>
       </c>
       <c r="V12" t="str">
-        <v>BP recorded at 154/96 mmHg in previous visit. Fasting blood sugar 184 mg/dL.</v>
+        <v>HbA1c: 8.8%. BP: 154/96 mmHg. Prescribed triple therapy.</v>
       </c>
       <c r="W12" t="str">
-        <v>Dr. S. K. Verma, MD</v>
+        <v>Dr. A. Gupta, MD</v>
       </c>
       <c r="X12" t="str">
-        <v/>
+        <v>Glycemic control suboptimal (HbA1c 8.8%). Advised dietary moderation and continued compliance.</v>
       </c>
       <c r="Y12" t="str">
         <v/>
       </c>
       <c r="Z12" t="str">
-        <v>Pending Verification</v>
+        <v>Verified by Doctor</v>
       </c>
       <c r="AA12" t="str">
-        <v/>
+        <v>2025-11-15</v>
       </c>
       <c r="AB12" t="str">
-        <v/>
+        <v>15:30:00</v>
       </c>
       <c r="AC12" t="str">
-        <v>Tab Ecosprin (Dispersible) (300 mg, Stat chewable, 1 day); Tab Clopidogrel (300 mg, Stat oral, 1 day); Tab Sorbitrate (Sublingual) (5 mg, SOS Sublingual, Stat); Tab Atorvastatin (80 mg, Stat bedtime, 1 day)</v>
+        <v>Telmisartan (40 mg, Once daily morning (1-0-0), 90 days); Metformin (500 mg, Twice daily (1-0-1), 90 days); Atorvastatin (20 mg, Once daily bedtime (0-0-1), 90 days)</v>
       </c>
       <c r="AD12" t="str">
-        <v>Tab Ecosprin (Dispersible)</v>
+        <v>Telmisartan</v>
       </c>
       <c r="AE12" t="str">
-        <v>300 mg</v>
+        <v>40 mg</v>
       </c>
       <c r="AF12" t="str">
-        <v>Stat chewable</v>
+        <v>Once daily morning (1-0-0)</v>
       </c>
       <c r="AG12" t="str">
-        <v>Chew immediately for acute coronary syndrome loading</v>
+        <v>Take in morning with water for blood pressure</v>
       </c>
       <c r="AH12" t="str">
         <v/>
@@ -1856,7 +1901,7 @@
         <v>Not Generated</v>
       </c>
       <c r="AJ12" t="str">
-        <v/>
+        <v>2025-11-15 15:30:00</v>
       </c>
       <c r="AK12" t="str">
         <v/>
@@ -1865,7 +1910,7 @@
         <v/>
       </c>
       <c r="AM12" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
     <row r="13">
@@ -1885,46 +1930,46 @@
         <v>9876543210</v>
       </c>
       <c r="F13" t="str">
-        <v>सीने में भारीपन व पसीना (Acute Chest Heaviness)</v>
+        <v>डायबिटीज और बीपी चेकअप (Diabetes &amp; BP Follow-up)</v>
       </c>
       <c r="G13" t="str">
-        <v>V002</v>
+        <v>V001</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-09-07</v>
+        <v>2025-11-15</v>
       </c>
       <c r="I13" t="str">
-        <v>19:32:43</v>
+        <v>15:00:00</v>
       </c>
       <c r="J13" t="str">
-        <v>2026-09-07</v>
+        <v>2025-11-15</v>
       </c>
       <c r="K13" t="str">
-        <v>19:32:43</v>
+        <v>15:00:00</v>
       </c>
       <c r="L13" t="str">
         <v>2025-11-15T09:00:00.000Z</v>
       </c>
       <c r="M13" t="str">
-        <v>2026-09-07T14:02:43.134Z</v>
+        <v>2025-11-15T09:30:00.000Z</v>
       </c>
       <c r="N13" t="str">
-        <v>undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined</v>
+        <v>रूटीन 3 महीने का चेकअप और दवाओं का रीफिल।</v>
       </c>
       <c r="O13" t="str">
-        <v>58-year-old male with prior hospital records (Visit 1, Nov 2025 for T2DM/HTN) returns with sudden onset crushing retrosternal chest heaviness since 2 hours. Pain radiates to left arm and shoulder, associated with severe cold diaphoresis. Prior medications documented: Metformin 500mg BD, Telmisartan 40mg OD, Atorvastatin 20mg HS.</v>
+        <v>58-year-old male attended for chronic disease monitoring. Reports compliance with oral hypoglycemics and antihypertensives. Recent HbA1c 8.8%.</v>
       </c>
       <c r="P13" t="str">
-        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2), Mixed Dyslipidemia</v>
+        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2)</v>
       </c>
       <c r="Q13" t="str">
         <v>Metformin 500 mg, Telmisartan 40 mg, Atorvastatin 20 mg, Aspirin (Enteric Coated) 75 mg</v>
       </c>
       <c r="R13" t="str">
-        <v>Penicillin (No known allergy)</v>
+        <v>Penicillin (No known adverse reaction)</v>
       </c>
       <c r="S13" t="str">
-        <v>Crushing retrosternal chest pain of acute onset radiating to left arm with profuse cold diaphoresis.; History of Uncontrolled Type 2 Diabetes (HbA1c 8.8%) and Essential Hypertension (BP 154/96 recorded in Nov 2025 visit).</v>
+        <v>None</v>
       </c>
       <c r="T13" t="str">
         <v>District_Civil_Hospital_Prescription_Nov2025.jpg (prescription)</v>
@@ -1933,40 +1978,40 @@
         <v>None</v>
       </c>
       <c r="V13" t="str">
-        <v>BP recorded at 154/96 mmHg in previous visit. Fasting blood sugar 184 mg/dL.</v>
+        <v>HbA1c: 8.8%. BP: 154/96 mmHg. Prescribed triple therapy.</v>
       </c>
       <c r="W13" t="str">
-        <v>Dr. S. K. Verma, MD</v>
+        <v>Dr. A. Gupta, MD</v>
       </c>
       <c r="X13" t="str">
-        <v/>
+        <v>Glycemic control suboptimal (HbA1c 8.8%). Advised dietary moderation and continued compliance.</v>
       </c>
       <c r="Y13" t="str">
         <v/>
       </c>
       <c r="Z13" t="str">
-        <v>Pending Verification</v>
+        <v>Verified by Doctor</v>
       </c>
       <c r="AA13" t="str">
-        <v/>
+        <v>2025-11-15</v>
       </c>
       <c r="AB13" t="str">
-        <v/>
+        <v>15:30:00</v>
       </c>
       <c r="AC13" t="str">
-        <v>Tab Ecosprin (Dispersible) (300 mg, Stat chewable, 1 day); Tab Clopidogrel (300 mg, Stat oral, 1 day); Tab Sorbitrate (Sublingual) (5 mg, SOS Sublingual, Stat); Tab Atorvastatin (80 mg, Stat bedtime, 1 day)</v>
+        <v>Telmisartan (40 mg, Once daily morning (1-0-0), 90 days); Metformin (500 mg, Twice daily (1-0-1), 90 days); Atorvastatin (20 mg, Once daily bedtime (0-0-1), 90 days)</v>
       </c>
       <c r="AD13" t="str">
-        <v>Tab Clopidogrel</v>
+        <v>Metformin</v>
       </c>
       <c r="AE13" t="str">
-        <v>300 mg</v>
+        <v>500 mg</v>
       </c>
       <c r="AF13" t="str">
-        <v>Stat oral</v>
+        <v>Twice daily (1-0-1)</v>
       </c>
       <c r="AG13" t="str">
-        <v>Loading dose taken immediately with water</v>
+        <v>Take after breakfast and dinner for blood sugar</v>
       </c>
       <c r="AH13" t="str">
         <v/>
@@ -1975,7 +2020,7 @@
         <v>Not Generated</v>
       </c>
       <c r="AJ13" t="str">
-        <v/>
+        <v>2025-11-15 15:30:00</v>
       </c>
       <c r="AK13" t="str">
         <v/>
@@ -1984,7 +2029,7 @@
         <v/>
       </c>
       <c r="AM13" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
     <row r="14">
@@ -2004,46 +2049,46 @@
         <v>9876543210</v>
       </c>
       <c r="F14" t="str">
-        <v>सीने में भारीपन व पसीना (Acute Chest Heaviness)</v>
+        <v>डायबिटीज और बीपी चेकअप (Diabetes &amp; BP Follow-up)</v>
       </c>
       <c r="G14" t="str">
-        <v>V002</v>
+        <v>V001</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-09-07</v>
+        <v>2025-11-15</v>
       </c>
       <c r="I14" t="str">
-        <v>19:32:43</v>
+        <v>15:00:00</v>
       </c>
       <c r="J14" t="str">
-        <v>2026-09-07</v>
+        <v>2025-11-15</v>
       </c>
       <c r="K14" t="str">
-        <v>19:32:43</v>
+        <v>15:00:00</v>
       </c>
       <c r="L14" t="str">
         <v>2025-11-15T09:00:00.000Z</v>
       </c>
       <c r="M14" t="str">
-        <v>2026-09-07T14:02:43.134Z</v>
+        <v>2025-11-15T09:30:00.000Z</v>
       </c>
       <c r="N14" t="str">
-        <v>undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined</v>
+        <v>रूटीन 3 महीने का चेकअप और दवाओं का रीफिल।</v>
       </c>
       <c r="O14" t="str">
-        <v>58-year-old male with prior hospital records (Visit 1, Nov 2025 for T2DM/HTN) returns with sudden onset crushing retrosternal chest heaviness since 2 hours. Pain radiates to left arm and shoulder, associated with severe cold diaphoresis. Prior medications documented: Metformin 500mg BD, Telmisartan 40mg OD, Atorvastatin 20mg HS.</v>
+        <v>58-year-old male attended for chronic disease monitoring. Reports compliance with oral hypoglycemics and antihypertensives. Recent HbA1c 8.8%.</v>
       </c>
       <c r="P14" t="str">
-        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2), Mixed Dyslipidemia</v>
+        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2)</v>
       </c>
       <c r="Q14" t="str">
         <v>Metformin 500 mg, Telmisartan 40 mg, Atorvastatin 20 mg, Aspirin (Enteric Coated) 75 mg</v>
       </c>
       <c r="R14" t="str">
-        <v>Penicillin (No known allergy)</v>
+        <v>Penicillin (No known adverse reaction)</v>
       </c>
       <c r="S14" t="str">
-        <v>Crushing retrosternal chest pain of acute onset radiating to left arm with profuse cold diaphoresis.; History of Uncontrolled Type 2 Diabetes (HbA1c 8.8%) and Essential Hypertension (BP 154/96 recorded in Nov 2025 visit).</v>
+        <v>None</v>
       </c>
       <c r="T14" t="str">
         <v>District_Civil_Hospital_Prescription_Nov2025.jpg (prescription)</v>
@@ -2052,40 +2097,40 @@
         <v>None</v>
       </c>
       <c r="V14" t="str">
-        <v>BP recorded at 154/96 mmHg in previous visit. Fasting blood sugar 184 mg/dL.</v>
+        <v>HbA1c: 8.8%. BP: 154/96 mmHg. Prescribed triple therapy.</v>
       </c>
       <c r="W14" t="str">
-        <v>Dr. S. K. Verma, MD</v>
+        <v>Dr. A. Gupta, MD</v>
       </c>
       <c r="X14" t="str">
-        <v/>
+        <v>Glycemic control suboptimal (HbA1c 8.8%). Advised dietary moderation and continued compliance.</v>
       </c>
       <c r="Y14" t="str">
         <v/>
       </c>
       <c r="Z14" t="str">
-        <v>Pending Verification</v>
+        <v>Verified by Doctor</v>
       </c>
       <c r="AA14" t="str">
-        <v/>
+        <v>2025-11-15</v>
       </c>
       <c r="AB14" t="str">
-        <v/>
+        <v>15:30:00</v>
       </c>
       <c r="AC14" t="str">
-        <v>Tab Ecosprin (Dispersible) (300 mg, Stat chewable, 1 day); Tab Clopidogrel (300 mg, Stat oral, 1 day); Tab Sorbitrate (Sublingual) (5 mg, SOS Sublingual, Stat); Tab Atorvastatin (80 mg, Stat bedtime, 1 day)</v>
+        <v>Telmisartan (40 mg, Once daily morning (1-0-0), 90 days); Metformin (500 mg, Twice daily (1-0-1), 90 days); Atorvastatin (20 mg, Once daily bedtime (0-0-1), 90 days)</v>
       </c>
       <c r="AD14" t="str">
-        <v>Tab Sorbitrate (Sublingual)</v>
+        <v>Atorvastatin</v>
       </c>
       <c r="AE14" t="str">
-        <v>5 mg</v>
+        <v>20 mg</v>
       </c>
       <c r="AF14" t="str">
-        <v>SOS Sublingual</v>
+        <v>Once daily bedtime (0-0-1)</v>
       </c>
       <c r="AG14" t="str">
-        <v>Place under tongue if chest heaviness recurs</v>
+        <v>Take at night for cholesterol control</v>
       </c>
       <c r="AH14" t="str">
         <v/>
@@ -2094,7 +2139,7 @@
         <v>Not Generated</v>
       </c>
       <c r="AJ14" t="str">
-        <v/>
+        <v>2025-11-15 15:30:00</v>
       </c>
       <c r="AK14" t="str">
         <v/>
@@ -2103,7 +2148,7 @@
         <v/>
       </c>
       <c r="AM14" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
     <row r="15">
@@ -2195,16 +2240,16 @@
         <v>Tab Ecosprin (Dispersible) (300 mg, Stat chewable, 1 day); Tab Clopidogrel (300 mg, Stat oral, 1 day); Tab Sorbitrate (Sublingual) (5 mg, SOS Sublingual, Stat); Tab Atorvastatin (80 mg, Stat bedtime, 1 day)</v>
       </c>
       <c r="AD15" t="str">
-        <v>Tab Atorvastatin</v>
+        <v>Tab Ecosprin (Dispersible)</v>
       </c>
       <c r="AE15" t="str">
-        <v>80 mg</v>
+        <v>300 mg</v>
       </c>
       <c r="AF15" t="str">
-        <v>Stat bedtime</v>
+        <v>Stat chewable</v>
       </c>
       <c r="AG15" t="str">
-        <v>High-intensity statin loading</v>
+        <v>Chew immediately for acute coronary syndrome loading</v>
       </c>
       <c r="AH15" t="str">
         <v/>
@@ -2222,250 +2267,607 @@
         <v/>
       </c>
       <c r="AM15" t="str">
-        <v>2026-09-09 10:52:33</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>P10027</v>
+        <v>P10026</v>
       </c>
       <c r="B16" t="str">
-        <v>Sunita Devi</v>
+        <v>Ramesh Kumar</v>
       </c>
       <c r="C16">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="D16" t="str">
-        <v>FEMALE</v>
+        <v>MALE</v>
       </c>
       <c r="E16" t="str">
-        <v>9845123670</v>
+        <v>9876543210</v>
       </c>
       <c r="F16" t="str">
-        <v>5 दिनों से तेज बुखार व कंपकंपी (High Grade Fever with Chills)</v>
+        <v>सीने में भारीपन व पसीना (Acute Chest Heaviness)</v>
       </c>
       <c r="G16" t="str">
-        <v>V001</v>
+        <v>V002</v>
       </c>
       <c r="H16" t="str">
         <v>2026-09-07</v>
       </c>
       <c r="I16" t="str">
-        <v>19:12:43</v>
+        <v>19:32:43</v>
       </c>
       <c r="J16" t="str">
         <v>2026-09-07</v>
       </c>
       <c r="K16" t="str">
-        <v>19:12:43</v>
+        <v>19:32:43</v>
       </c>
       <c r="L16" t="str">
-        <v>2026-09-07T08:30:00.000Z</v>
+        <v>2025-11-15T09:00:00.000Z</v>
       </c>
       <c r="M16" t="str">
-        <v>2026-09-07T13:42:43.135Z</v>
+        <v>2026-09-07T14:02:43.134Z</v>
       </c>
       <c r="N16" t="str">
-        <v>undefined: undefined; undefined: undefined; undefined: undefined</v>
+        <v>undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined</v>
       </c>
       <c r="O16" t="str">
-        <v>42-year-old female presents with 5-day history of acute high-grade fever accompanied by severe chills, retro-orbital ache, and generalized myalgia. Uploaded NABL lab report dated 18-Feb-2026 confirms Dengue NS1 Antigen Reactive with critical Platelet count of 58,000 /uL.</v>
+        <v>58-year-old male with prior hospital records (Visit 1, Nov 2025 for T2DM/HTN) returns with sudden onset crushing retrosternal chest heaviness since 2 hours. Pain radiates to left arm and shoulder, associated with severe cold diaphoresis. Prior medications documented: Metformin 500mg BD, Telmisartan 40mg OD, Atorvastatin 20mg HS.</v>
       </c>
       <c r="P16" t="str">
-        <v>Type-2 Diabetes (HbA1c 9.2% detected on recent panel)</v>
+        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2), Mixed Dyslipidemia</v>
       </c>
       <c r="Q16" t="str">
-        <v>None</v>
+        <v>Metformin 500 mg, Telmisartan 40 mg, Atorvastatin 20 mg, Aspirin (Enteric Coated) 75 mg</v>
       </c>
       <c r="R16" t="str">
-        <v>NSAIDs (Diclofenac/Ibuprofen) (Avoid strictly due to bleeding risk in Dengue)</v>
+        <v>Penicillin (No known allergy)</v>
       </c>
       <c r="S16" t="str">
-        <v>Platelet count 58,000/uL with mucosal bleeding (epistaxis/gingival bleeding).</v>
+        <v>Crushing retrosternal chest pain of acute onset radiating to left arm with profuse cold diaphoresis.; History of Uncontrolled Type 2 Diabetes (HbA1c 8.8%) and Essential Hypertension (BP 154/96 recorded in Nov 2025 visit).</v>
       </c>
       <c r="T16" t="str">
-        <v>National_Lab_Hematology_Feb2026.pdf (lab_report)</v>
+        <v>District_Civil_Hospital_Prescription_Nov2025.jpg (prescription)</v>
       </c>
       <c r="U16" t="str">
         <v>None</v>
       </c>
       <c r="V16" t="str">
-        <v>Patient admitted for dengue monitoring.</v>
+        <v>BP recorded at 154/96 mmHg in previous visit. Fasting blood sugar 184 mg/dL.</v>
       </c>
       <c r="W16" t="str">
         <v>Dr. S. K. Verma, MD</v>
       </c>
       <c r="X16" t="str">
-        <v>Patient admitted for dengue monitoring.</v>
+        <v/>
       </c>
       <c r="Y16" t="str">
         <v/>
       </c>
       <c r="Z16" t="str">
-        <v>Verified by Doctor</v>
+        <v>Pending Verification</v>
       </c>
       <c r="AA16" t="str">
-        <v>2026-09-07</v>
+        <v/>
       </c>
       <c r="AB16" t="str">
-        <v>22:40:16</v>
+        <v/>
       </c>
       <c r="AC16" t="str">
-        <v>Tab Paracetamol (650 mg, 1-1-1-1 (TDS/QID SOS), 5 days); Sachet ORS (Oral Rehydration Salts) (1 Packet in 1L water, Sip frequently, 5 days)</v>
+        <v>Tab Ecosprin (Dispersible) (300 mg, Stat chewable, 1 day); Tab Clopidogrel (300 mg, Stat oral, 1 day); Tab Sorbitrate (Sublingual) (5 mg, SOS Sublingual, Stat); Tab Atorvastatin (80 mg, Stat bedtime, 1 day)</v>
       </c>
       <c r="AD16" t="str">
-        <v>Tab Paracetamol</v>
+        <v>Tab Clopidogrel</v>
       </c>
       <c r="AE16" t="str">
-        <v>650 mg</v>
+        <v>300 mg</v>
       </c>
       <c r="AF16" t="str">
-        <v>1-1-1-1 (TDS/QID SOS)</v>
+        <v>Stat oral</v>
       </c>
       <c r="AG16" t="str">
-        <v>Take only for fever &gt; 100°F. STRICTLY AVOID NSAIDs / BRUFEN</v>
+        <v>Loading dose taken immediately with water</v>
       </c>
       <c r="AH16" t="str">
         <v/>
       </c>
       <c r="AI16" t="str">
-        <v>Generated</v>
+        <v>Not Generated</v>
       </c>
       <c r="AJ16" t="str">
-        <v>2026-09-07 22:40:16</v>
+        <v/>
       </c>
       <c r="AK16" t="str">
-        <v>http://localhost:5173/receipt/ac507d7c187c806b1acc8273f9ed35935091810fda0aeda3</v>
+        <v/>
       </c>
       <c r="AL16" t="str">
         <v/>
       </c>
       <c r="AM16" t="str">
-        <v>2026-09-07 22:40:16</v>
+        <v>2026-09-10 10:52:34</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>P10027</v>
+        <v>P10026</v>
       </c>
       <c r="B17" t="str">
-        <v>Sunita Devi</v>
+        <v>Ramesh Kumar</v>
       </c>
       <c r="C17">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="D17" t="str">
-        <v>FEMALE</v>
+        <v>MALE</v>
       </c>
       <c r="E17" t="str">
-        <v>9845123670</v>
+        <v>9876543210</v>
       </c>
       <c r="F17" t="str">
-        <v>5 दिनों से तेज बुखार व कंपकंपी (High Grade Fever with Chills)</v>
+        <v>सीने में भारीपन व पसीना (Acute Chest Heaviness)</v>
       </c>
       <c r="G17" t="str">
-        <v>V001</v>
+        <v>V002</v>
       </c>
       <c r="H17" t="str">
         <v>2026-09-07</v>
       </c>
       <c r="I17" t="str">
-        <v>19:12:43</v>
+        <v>19:32:43</v>
       </c>
       <c r="J17" t="str">
         <v>2026-09-07</v>
       </c>
       <c r="K17" t="str">
-        <v>19:12:43</v>
+        <v>19:32:43</v>
       </c>
       <c r="L17" t="str">
-        <v>2026-09-07T08:30:00.000Z</v>
+        <v>2025-11-15T09:00:00.000Z</v>
       </c>
       <c r="M17" t="str">
-        <v>2026-09-07T13:42:43.135Z</v>
+        <v>2026-09-07T14:02:43.134Z</v>
       </c>
       <c r="N17" t="str">
-        <v>undefined: undefined; undefined: undefined; undefined: undefined</v>
+        <v>undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined</v>
       </c>
       <c r="O17" t="str">
-        <v>42-year-old female presents with 5-day history of acute high-grade fever accompanied by severe chills, retro-orbital ache, and generalized myalgia. Uploaded NABL lab report dated 18-Feb-2026 confirms Dengue NS1 Antigen Reactive with critical Platelet count of 58,000 /uL.</v>
+        <v>58-year-old male with prior hospital records (Visit 1, Nov 2025 for T2DM/HTN) returns with sudden onset crushing retrosternal chest heaviness since 2 hours. Pain radiates to left arm and shoulder, associated with severe cold diaphoresis. Prior medications documented: Metformin 500mg BD, Telmisartan 40mg OD, Atorvastatin 20mg HS.</v>
       </c>
       <c r="P17" t="str">
-        <v>Type-2 Diabetes (HbA1c 9.2% detected on recent panel)</v>
+        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2), Mixed Dyslipidemia</v>
       </c>
       <c r="Q17" t="str">
-        <v>None</v>
+        <v>Metformin 500 mg, Telmisartan 40 mg, Atorvastatin 20 mg, Aspirin (Enteric Coated) 75 mg</v>
       </c>
       <c r="R17" t="str">
-        <v>NSAIDs (Diclofenac/Ibuprofen) (Avoid strictly due to bleeding risk in Dengue)</v>
+        <v>Penicillin (No known allergy)</v>
       </c>
       <c r="S17" t="str">
-        <v>Platelet count 58,000/uL with mucosal bleeding (epistaxis/gingival bleeding).</v>
+        <v>Crushing retrosternal chest pain of acute onset radiating to left arm with profuse cold diaphoresis.; History of Uncontrolled Type 2 Diabetes (HbA1c 8.8%) and Essential Hypertension (BP 154/96 recorded in Nov 2025 visit).</v>
       </c>
       <c r="T17" t="str">
-        <v>National_Lab_Hematology_Feb2026.pdf (lab_report)</v>
+        <v>District_Civil_Hospital_Prescription_Nov2025.jpg (prescription)</v>
       </c>
       <c r="U17" t="str">
         <v>None</v>
       </c>
       <c r="V17" t="str">
-        <v>Patient admitted for dengue monitoring.</v>
+        <v>BP recorded at 154/96 mmHg in previous visit. Fasting blood sugar 184 mg/dL.</v>
       </c>
       <c r="W17" t="str">
         <v>Dr. S. K. Verma, MD</v>
       </c>
       <c r="X17" t="str">
+        <v/>
+      </c>
+      <c r="Y17" t="str">
+        <v/>
+      </c>
+      <c r="Z17" t="str">
+        <v>Pending Verification</v>
+      </c>
+      <c r="AA17" t="str">
+        <v/>
+      </c>
+      <c r="AB17" t="str">
+        <v/>
+      </c>
+      <c r="AC17" t="str">
+        <v>Tab Ecosprin (Dispersible) (300 mg, Stat chewable, 1 day); Tab Clopidogrel (300 mg, Stat oral, 1 day); Tab Sorbitrate (Sublingual) (5 mg, SOS Sublingual, Stat); Tab Atorvastatin (80 mg, Stat bedtime, 1 day)</v>
+      </c>
+      <c r="AD17" t="str">
+        <v>Tab Sorbitrate (Sublingual)</v>
+      </c>
+      <c r="AE17" t="str">
+        <v>5 mg</v>
+      </c>
+      <c r="AF17" t="str">
+        <v>SOS Sublingual</v>
+      </c>
+      <c r="AG17" t="str">
+        <v>Place under tongue if chest heaviness recurs</v>
+      </c>
+      <c r="AH17" t="str">
+        <v/>
+      </c>
+      <c r="AI17" t="str">
+        <v>Not Generated</v>
+      </c>
+      <c r="AJ17" t="str">
+        <v/>
+      </c>
+      <c r="AK17" t="str">
+        <v/>
+      </c>
+      <c r="AL17" t="str">
+        <v/>
+      </c>
+      <c r="AM17" t="str">
+        <v>2026-09-10 10:52:34</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>P10026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Ramesh Kumar</v>
+      </c>
+      <c r="C18">
+        <v>58</v>
+      </c>
+      <c r="D18" t="str">
+        <v>MALE</v>
+      </c>
+      <c r="E18" t="str">
+        <v>9876543210</v>
+      </c>
+      <c r="F18" t="str">
+        <v>सीने में भारीपन व पसीना (Acute Chest Heaviness)</v>
+      </c>
+      <c r="G18" t="str">
+        <v>V002</v>
+      </c>
+      <c r="H18" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="I18" t="str">
+        <v>19:32:43</v>
+      </c>
+      <c r="J18" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="K18" t="str">
+        <v>19:32:43</v>
+      </c>
+      <c r="L18" t="str">
+        <v>2025-11-15T09:00:00.000Z</v>
+      </c>
+      <c r="M18" t="str">
+        <v>2026-09-07T14:02:43.134Z</v>
+      </c>
+      <c r="N18" t="str">
+        <v>undefined: undefined; undefined: undefined; undefined: undefined; undefined: undefined</v>
+      </c>
+      <c r="O18" t="str">
+        <v>58-year-old male with prior hospital records (Visit 1, Nov 2025 for T2DM/HTN) returns with sudden onset crushing retrosternal chest heaviness since 2 hours. Pain radiates to left arm and shoulder, associated with severe cold diaphoresis. Prior medications documented: Metformin 500mg BD, Telmisartan 40mg OD, Atorvastatin 20mg HS.</v>
+      </c>
+      <c r="P18" t="str">
+        <v>Type 2 Diabetes Mellitus (Uncontrolled), Essential Hypertension (Stage 2), Mixed Dyslipidemia</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>Metformin 500 mg, Telmisartan 40 mg, Atorvastatin 20 mg, Aspirin (Enteric Coated) 75 mg</v>
+      </c>
+      <c r="R18" t="str">
+        <v>Penicillin (No known allergy)</v>
+      </c>
+      <c r="S18" t="str">
+        <v>Crushing retrosternal chest pain of acute onset radiating to left arm with profuse cold diaphoresis.; History of Uncontrolled Type 2 Diabetes (HbA1c 8.8%) and Essential Hypertension (BP 154/96 recorded in Nov 2025 visit).</v>
+      </c>
+      <c r="T18" t="str">
+        <v>District_Civil_Hospital_Prescription_Nov2025.jpg (prescription)</v>
+      </c>
+      <c r="U18" t="str">
+        <v>None</v>
+      </c>
+      <c r="V18" t="str">
+        <v>BP recorded at 154/96 mmHg in previous visit. Fasting blood sugar 184 mg/dL.</v>
+      </c>
+      <c r="W18" t="str">
+        <v>Dr. S. K. Verma, MD</v>
+      </c>
+      <c r="X18" t="str">
+        <v/>
+      </c>
+      <c r="Y18" t="str">
+        <v/>
+      </c>
+      <c r="Z18" t="str">
+        <v>Pending Verification</v>
+      </c>
+      <c r="AA18" t="str">
+        <v/>
+      </c>
+      <c r="AB18" t="str">
+        <v/>
+      </c>
+      <c r="AC18" t="str">
+        <v>Tab Ecosprin (Dispersible) (300 mg, Stat chewable, 1 day); Tab Clopidogrel (300 mg, Stat oral, 1 day); Tab Sorbitrate (Sublingual) (5 mg, SOS Sublingual, Stat); Tab Atorvastatin (80 mg, Stat bedtime, 1 day)</v>
+      </c>
+      <c r="AD18" t="str">
+        <v>Tab Atorvastatin</v>
+      </c>
+      <c r="AE18" t="str">
+        <v>80 mg</v>
+      </c>
+      <c r="AF18" t="str">
+        <v>Stat bedtime</v>
+      </c>
+      <c r="AG18" t="str">
+        <v>High-intensity statin loading</v>
+      </c>
+      <c r="AH18" t="str">
+        <v/>
+      </c>
+      <c r="AI18" t="str">
+        <v>Not Generated</v>
+      </c>
+      <c r="AJ18" t="str">
+        <v/>
+      </c>
+      <c r="AK18" t="str">
+        <v/>
+      </c>
+      <c r="AL18" t="str">
+        <v/>
+      </c>
+      <c r="AM18" t="str">
+        <v>2026-09-10 10:52:34</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>P10027</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Sunita Devi</v>
+      </c>
+      <c r="C19">
+        <v>42</v>
+      </c>
+      <c r="D19" t="str">
+        <v>FEMALE</v>
+      </c>
+      <c r="E19" t="str">
+        <v>9845123670</v>
+      </c>
+      <c r="F19" t="str">
+        <v>5 दिनों से तेज बुखार व कंपकंपी (High Grade Fever with Chills)</v>
+      </c>
+      <c r="G19" t="str">
+        <v>V001</v>
+      </c>
+      <c r="H19" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="I19" t="str">
+        <v>19:12:43</v>
+      </c>
+      <c r="J19" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="K19" t="str">
+        <v>19:12:43</v>
+      </c>
+      <c r="L19" t="str">
+        <v>2026-09-07T08:30:00.000Z</v>
+      </c>
+      <c r="M19" t="str">
+        <v>2026-09-07T13:42:43.135Z</v>
+      </c>
+      <c r="N19" t="str">
+        <v>undefined: undefined; undefined: undefined; undefined: undefined</v>
+      </c>
+      <c r="O19" t="str">
+        <v>42-year-old female presents with 5-day history of acute high-grade fever accompanied by severe chills, retro-orbital ache, and generalized myalgia. Uploaded NABL lab report dated 18-Feb-2026 confirms Dengue NS1 Antigen Reactive with critical Platelet count of 58,000 /uL.</v>
+      </c>
+      <c r="P19" t="str">
+        <v>Type-2 Diabetes (HbA1c 9.2% detected on recent panel)</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>None</v>
+      </c>
+      <c r="R19" t="str">
+        <v>NSAIDs (Diclofenac/Ibuprofen) (Avoid strictly due to bleeding risk in Dengue)</v>
+      </c>
+      <c r="S19" t="str">
+        <v>Platelet count 58,000/uL with mucosal bleeding (epistaxis/gingival bleeding).</v>
+      </c>
+      <c r="T19" t="str">
+        <v>National_Lab_Hematology_Feb2026.pdf (lab_report)</v>
+      </c>
+      <c r="U19" t="str">
+        <v>None</v>
+      </c>
+      <c r="V19" t="str">
         <v>Patient admitted for dengue monitoring.</v>
       </c>
-      <c r="Y17" t="str">
-        <v/>
-      </c>
-      <c r="Z17" t="str">
+      <c r="W19" t="str">
+        <v>Dr. S. K. Verma, MD</v>
+      </c>
+      <c r="X19" t="str">
+        <v>Patient admitted for dengue monitoring.</v>
+      </c>
+      <c r="Y19" t="str">
+        <v/>
+      </c>
+      <c r="Z19" t="str">
         <v>Verified by Doctor</v>
       </c>
-      <c r="AA17" t="str">
+      <c r="AA19" t="str">
         <v>2026-09-07</v>
       </c>
-      <c r="AB17" t="str">
+      <c r="AB19" t="str">
         <v>22:40:16</v>
       </c>
-      <c r="AC17" t="str">
+      <c r="AC19" t="str">
         <v>Tab Paracetamol (650 mg, 1-1-1-1 (TDS/QID SOS), 5 days); Sachet ORS (Oral Rehydration Salts) (1 Packet in 1L water, Sip frequently, 5 days)</v>
       </c>
-      <c r="AD17" t="str">
+      <c r="AD19" t="str">
+        <v>Tab Paracetamol</v>
+      </c>
+      <c r="AE19" t="str">
+        <v>650 mg</v>
+      </c>
+      <c r="AF19" t="str">
+        <v>1-1-1-1 (TDS/QID SOS)</v>
+      </c>
+      <c r="AG19" t="str">
+        <v>Take only for fever &gt; 100°F. STRICTLY AVOID NSAIDs / BRUFEN</v>
+      </c>
+      <c r="AH19" t="str">
+        <v/>
+      </c>
+      <c r="AI19" t="str">
+        <v>Generated</v>
+      </c>
+      <c r="AJ19" t="str">
+        <v>2026-09-07 22:40:16</v>
+      </c>
+      <c r="AK19" t="str">
+        <v>http://localhost:5173/receipt/ac507d7c187c806b1acc8273f9ed35935091810fda0aeda3</v>
+      </c>
+      <c r="AL19" t="str">
+        <v/>
+      </c>
+      <c r="AM19" t="str">
+        <v>2026-09-07 22:40:16</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>P10027</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Sunita Devi</v>
+      </c>
+      <c r="C20">
+        <v>42</v>
+      </c>
+      <c r="D20" t="str">
+        <v>FEMALE</v>
+      </c>
+      <c r="E20" t="str">
+        <v>9845123670</v>
+      </c>
+      <c r="F20" t="str">
+        <v>5 दिनों से तेज बुखार व कंपकंपी (High Grade Fever with Chills)</v>
+      </c>
+      <c r="G20" t="str">
+        <v>V001</v>
+      </c>
+      <c r="H20" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="I20" t="str">
+        <v>19:12:43</v>
+      </c>
+      <c r="J20" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="K20" t="str">
+        <v>19:12:43</v>
+      </c>
+      <c r="L20" t="str">
+        <v>2026-09-07T08:30:00.000Z</v>
+      </c>
+      <c r="M20" t="str">
+        <v>2026-09-07T13:42:43.135Z</v>
+      </c>
+      <c r="N20" t="str">
+        <v>undefined: undefined; undefined: undefined; undefined: undefined</v>
+      </c>
+      <c r="O20" t="str">
+        <v>42-year-old female presents with 5-day history of acute high-grade fever accompanied by severe chills, retro-orbital ache, and generalized myalgia. Uploaded NABL lab report dated 18-Feb-2026 confirms Dengue NS1 Antigen Reactive with critical Platelet count of 58,000 /uL.</v>
+      </c>
+      <c r="P20" t="str">
+        <v>Type-2 Diabetes (HbA1c 9.2% detected on recent panel)</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>None</v>
+      </c>
+      <c r="R20" t="str">
+        <v>NSAIDs (Diclofenac/Ibuprofen) (Avoid strictly due to bleeding risk in Dengue)</v>
+      </c>
+      <c r="S20" t="str">
+        <v>Platelet count 58,000/uL with mucosal bleeding (epistaxis/gingival bleeding).</v>
+      </c>
+      <c r="T20" t="str">
+        <v>National_Lab_Hematology_Feb2026.pdf (lab_report)</v>
+      </c>
+      <c r="U20" t="str">
+        <v>None</v>
+      </c>
+      <c r="V20" t="str">
+        <v>Patient admitted for dengue monitoring.</v>
+      </c>
+      <c r="W20" t="str">
+        <v>Dr. S. K. Verma, MD</v>
+      </c>
+      <c r="X20" t="str">
+        <v>Patient admitted for dengue monitoring.</v>
+      </c>
+      <c r="Y20" t="str">
+        <v/>
+      </c>
+      <c r="Z20" t="str">
+        <v>Verified by Doctor</v>
+      </c>
+      <c r="AA20" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="AB20" t="str">
+        <v>22:40:16</v>
+      </c>
+      <c r="AC20" t="str">
+        <v>Tab Paracetamol (650 mg, 1-1-1-1 (TDS/QID SOS), 5 days); Sachet ORS (Oral Rehydration Salts) (1 Packet in 1L water, Sip frequently, 5 days)</v>
+      </c>
+      <c r="AD20" t="str">
         <v>Sachet ORS (Oral Rehydration Salts)</v>
       </c>
-      <c r="AE17" t="str">
+      <c r="AE20" t="str">
         <v>1 Packet in 1L water</v>
       </c>
-      <c r="AF17" t="str">
+      <c r="AF20" t="str">
         <v>Sip frequently</v>
       </c>
-      <c r="AG17" t="str">
+      <c r="AG20" t="str">
         <v>Drink 2.5 to 3 Litres of fluids daily</v>
       </c>
-      <c r="AH17" t="str">
-        <v/>
-      </c>
-      <c r="AI17" t="str">
+      <c r="AH20" t="str">
+        <v/>
+      </c>
+      <c r="AI20" t="str">
         <v>Generated</v>
       </c>
-      <c r="AJ17" t="str">
+      <c r="AJ20" t="str">
         <v>2026-09-07 22:40:16</v>
       </c>
-      <c r="AK17" t="str">
+      <c r="AK20" t="str">
         <v>http://localhost:5173/receipt/ac507d7c187c806b1acc8273f9ed35935091810fda0aeda3</v>
       </c>
-      <c r="AL17" t="str">
-        <v/>
-      </c>
-      <c r="AM17" t="str">
+      <c r="AL20" t="str">
+        <v/>
+      </c>
+      <c r="AM20" t="str">
         <v>2026-09-07 22:40:16</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AM17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AM20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>